<commit_message>
Commit on 18-02-2026 06:08PM
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/APITestData.xlsx
+++ b/src/test/resources/testdata/APITestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\APIAutomationFramework\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B41DD7C-FDBD-4354-96D4-E945A2772A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC374B2B-4354-4ED1-831A-C7038CA7ED50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-100" yWindow="-100" windowWidth="21467" windowHeight="11443" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-100" yWindow="-100" windowWidth="21467" windowHeight="11443" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GetPetsAPI" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>UserName</t>
   </si>
@@ -448,8 +448,8 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>5555</v>
+      <c r="A2" t="s">
+        <v>13</v>
       </c>
       <c r="B2">
         <v>200</v>
@@ -459,11 +459,11 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>6565</v>
+      <c r="A3" t="s">
+        <v>20</v>
       </c>
       <c r="B3">
-        <v>404</v>
+        <v>200</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>

</xml_diff>